<commit_message>
Extract INE Venezuela tabular values
</commit_message>
<xml_diff>
--- a/assets/data/ine/catalog/catalogo_dataset_web_ove_ine_venezuela.xlsx
+++ b/assets/data/ine/catalog/catalogo_dataset_web_ove_ine_venezuela.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="catalogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="metadatos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="catalogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metadatos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -88,79 +88,11 @@
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -175,13 +107,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -190,7 +122,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -205,13 +137,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -19021,7 +18953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -19159,6 +19091,38 @@
         <v>119</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Hojas extraídas</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Celdas con valor extraídas</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>2980320</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Archivo valores CSV.GZ</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>assets/data/ine/csv/ove_ine_venezuela_celdas_tabulares.csv.gz</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>